<commit_message>
feat(kaggle-experiments): Add 3 specialized Kaggle notebooks for Dual T4 GPU training across 3 accounts (PPE 3-class, Color Helmet 5-class, Full 6-class master)
</commit_message>
<xml_diff>
--- a/AI_Capstone_Review123_Template_backup.xlsx
+++ b/AI_Capstone_Review123_Template_backup.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="69">
   <si>
     <r>
       <rPr>
@@ -76,14 +76,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
       <t>Thời gian</t>
     </r>
     <r>
@@ -258,6 +250,28 @@
         <charset val="134"/>
       </rPr>
       <t xml:space="preserve"> : </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Thời gian</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>:</t>
     </r>
   </si>
   <si>
@@ -423,6 +437,14 @@
       <i/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -575,14 +597,6 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="34">
@@ -1007,133 +1021,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1194,6 +1208,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1207,11 +1224,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1701,7 +1715,7 @@
     <col min="8" max="26" width="8.71296296296296" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7">
+    <row r="3" ht="14.4" spans="2:7">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1712,7 +1726,7 @@
       </c>
     </row>
     <row r="5" spans="2:7">
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="26" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1723,28 +1737,28 @@
       <c r="C7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="28"/>
+      <c r="G7" s="29"/>
     </row>
     <row r="8" ht="34.5" customHeight="1" spans="2:7">
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="30" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="28" t="s">
+      <c r="G8" s="29" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1771,10 +1785,10 @@
       <c r="D10" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="29" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1786,10 +1800,10 @@
       <c r="D11" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="28" t="s">
+      <c r="G11" s="29" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1808,16 +1822,16 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="2:7">
+    <row r="13" ht="14.4" spans="2:7">
       <c r="B13" s="8"/>
       <c r="C13" s="34" t="s">
         <v>28</v>
       </c>
       <c r="D13" s="31"/>
-      <c r="F13" s="28" t="s">
+      <c r="F13" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="28" t="s">
+      <c r="G13" s="29" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2906,7 +2920,7 @@
     </row>
     <row r="5" ht="14.4" spans="2:4">
       <c r="B5" s="1" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1" spans="2:4">
@@ -2922,63 +2936,63 @@
     </row>
     <row r="8" ht="31.5" customHeight="1" spans="2:4">
       <c r="B8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="5"/>
     </row>
     <row r="9" ht="31.5" customHeight="1" spans="2:4">
       <c r="B9" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D9" s="5"/>
     </row>
     <row r="10" ht="31.5" customHeight="1" spans="2:4">
       <c r="B10" s="8"/>
       <c r="C10" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10" s="5"/>
     </row>
     <row r="11" ht="31.5" customHeight="1" spans="2:4">
       <c r="B11" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
     </row>
     <row r="12" ht="14.4" spans="2:4">
       <c r="B12" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D12" s="13"/>
     </row>
     <row r="13" ht="43.2" spans="2:4">
       <c r="B13" s="14"/>
       <c r="C13" s="34" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" s="13"/>
     </row>
     <row r="14" ht="28.8" spans="2:4">
       <c r="B14" s="14"/>
       <c r="C14" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" ht="28.8" spans="2:4">
       <c r="B15" s="14"/>
       <c r="C15" s="34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D15" s="13"/>
     </row>
@@ -2991,31 +3005,31 @@
     </row>
     <row r="17" ht="48.75" customHeight="1" spans="2:4">
       <c r="B17" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" ht="48.75" customHeight="1" spans="2:4">
       <c r="B18" s="14"/>
       <c r="C18" s="34" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D18" s="13"/>
     </row>
     <row r="19" ht="48.75" customHeight="1" spans="2:4">
       <c r="B19" s="14"/>
       <c r="C19" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D19" s="13"/>
     </row>
     <row r="20" ht="48.75" customHeight="1" spans="2:4">
       <c r="B20" s="14"/>
       <c r="C20" s="34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D20" s="13"/>
     </row>
@@ -3028,31 +3042,31 @@
     </row>
     <row r="22" ht="48.75" customHeight="1" spans="2:4">
       <c r="B22" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="13"/>
     </row>
     <row r="23" ht="48.75" customHeight="1" spans="2:4">
       <c r="B23" s="14"/>
       <c r="C23" s="34" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D23" s="13"/>
     </row>
     <row r="24" ht="48.75" customHeight="1" spans="2:4">
       <c r="B24" s="14"/>
       <c r="C24" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D24" s="13"/>
     </row>
     <row r="25" ht="48.75" customHeight="1" spans="2:4">
       <c r="B25" s="14"/>
       <c r="C25" s="34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D25" s="13"/>
     </row>
@@ -4087,7 +4101,7 @@
     </row>
     <row r="5" ht="14.4" spans="2:4">
       <c r="B5" s="1" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1" spans="2:4">
@@ -4103,63 +4117,63 @@
     </row>
     <row r="8" ht="28.8" spans="2:4">
       <c r="B8" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D8" s="5"/>
     </row>
     <row r="9" ht="31.5" hidden="1" customHeight="1" spans="2:4">
       <c r="B9" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" ht="31.5" hidden="1" customHeight="1" spans="2:4">
       <c r="B10" s="8"/>
       <c r="C10" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" ht="31.5" customHeight="1" spans="2:4">
       <c r="B11" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
     </row>
     <row r="12" ht="48.75" customHeight="1" spans="2:4">
       <c r="B12" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D12" s="13"/>
     </row>
     <row r="13" ht="48.75" customHeight="1" spans="2:4">
       <c r="B13" s="14"/>
       <c r="C13" s="34" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" s="13"/>
     </row>
     <row r="14" ht="48.75" customHeight="1" spans="2:4">
       <c r="B14" s="14"/>
       <c r="C14" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" ht="48.75" customHeight="1" spans="2:4">
       <c r="B15" s="14"/>
       <c r="C15" s="34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D15" s="13"/>
     </row>
@@ -4172,31 +4186,31 @@
     </row>
     <row r="17" ht="48.75" customHeight="1" spans="1:26">
       <c r="B17" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" ht="48.75" customHeight="1" spans="1:26">
       <c r="B18" s="14"/>
       <c r="C18" s="34" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D18" s="13"/>
     </row>
     <row r="19" ht="48.75" customHeight="1" spans="1:26">
       <c r="B19" s="14"/>
       <c r="C19" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D19" s="13"/>
     </row>
     <row r="20" ht="48.75" customHeight="1" spans="1:26">
       <c r="B20" s="14"/>
       <c r="C20" s="34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D20" s="13"/>
     </row>
@@ -4209,31 +4223,31 @@
     </row>
     <row r="22" ht="48.75" customHeight="1" spans="1:26">
       <c r="B22" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C22" s="34" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="13"/>
     </row>
     <row r="23" ht="48.75" customHeight="1" spans="1:26">
       <c r="B23" s="14"/>
       <c r="C23" s="34" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D23" s="13"/>
     </row>
     <row r="24" ht="48.75" customHeight="1" spans="1:26">
       <c r="B24" s="14"/>
       <c r="C24" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D24" s="13"/>
     </row>
     <row r="25" ht="48.75" customHeight="1" spans="1:26">
       <c r="B25" s="14"/>
       <c r="C25" s="34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D25" s="13"/>
     </row>
@@ -4246,28 +4260,28 @@
     </row>
     <row r="27" ht="33.75" customHeight="1" spans="1:26">
       <c r="B27" s="15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
     </row>
     <row r="28" ht="14.4" spans="1:26">
       <c r="B28" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:26">
       <c r="B29" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:26">
       <c r="A30" s="19"/>
       <c r="B30" s="20"/>
       <c r="C30" s="21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D30" s="19"/>
       <c r="E30" s="19"/>
@@ -4295,25 +4309,25 @@
     </row>
     <row r="31" ht="32.25" customHeight="1" spans="1:26">
       <c r="B31" s="22" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C31" s="23"/>
     </row>
     <row r="32" ht="32.25" customHeight="1" spans="1:26">
       <c r="B32" s="22" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C32" s="23"/>
     </row>
     <row r="33" ht="32.25" customHeight="1" spans="2:3">
       <c r="B33" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C33" s="23"/>
     </row>
     <row r="34" ht="32.25" customHeight="1" spans="2:3">
       <c r="B34" s="24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C34" s="23"/>
     </row>

</xml_diff>